<commit_message>
B6 deal load list: record Option A, 500% approval and PBDD status
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECNUyLvUafHehET6NevFNz
</commit_message>
<xml_diff>
--- a/docs/deals/B6_Deal_PPC_Load_List_20260926.xlsx
+++ b/docs/deals/B6_Deal_PPC_Load_List_20260926.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +39,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
     </font>
   </fonts>
   <fills count="5">
@@ -76,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -87,6 +91,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -452,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="170" customWidth="1" min="1" max="1"/>
@@ -466,70 +474,77 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Built from run 20260924-981b2555, the B6 corrections document, Joseph’s pre-deal plan (built 23 Sep) and Command Center reads to 23 Sep. Deal prices from Umair’s sheet (10% off: King $76.49, Queen $71.99, Full $62.99).</t>
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>DECISIONS 26 Sep: Out of focus = OPTION A (flagship flat; +10% top-of-search test for two weeks on the converters, capped at the deal stop; read 10 Oct) — upload the Option A bulk file, NOT Option B. Modifiers over 500% APPROVED (operator sign-off 26 Sep). Prime Big Deal Days (7–8 Oct): not decided yet.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HOW TO USE: 1) Pull every row on the “Pull before loading” sheet. 2) Confirm the enrolled list (Queen Creme, King Taupe, Twin Sage Green, Cal King White). 3) Take the Decisions sheet to Erik/Joseph. 4) Load the Push list from LIVE values: re-read each campaign’s base and modifier, apply the step %, and never go above the “Deal stop” price.</t>
+          <t>Built from run 20260924-981b2555, the B6 corrections document, Joseph’s pre-deal plan (built 23 Sep) and Command Center reads to 23 Sep. Deal prices from Umair’s sheet (10% off: King $76.49, Queen $71.99, Full $62.99).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Prices here are from the audit read (24 Sep). The engine moved 15 bids and modifiers on 24 Sep after the audit, so where the live price differs, apply the step % to the live price and cap at the stop.</t>
+          <t>HOW TO USE: 1) Pull every row on the “Pull before loading” sheet. 2) Confirm the enrolled list (Queen Creme, King Taupe, Twin Sage Green, Cal King White). 3) Take the Decisions sheet to Erik/Joseph. 4) Load the Push list from LIVE values: re-read each campaign’s base and modifier, apply the step %, and never go above the “Deal stop” price.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Deal stop = 3 × deal contribution × the campaign’s top-of-search conversion rate (the corrections doc’s loss stop, recomputed at the deal price). Deal contribution = deal price − 15% referral − FBA fee − landed cost (Command Center economics); Amazon’s deal fee (~$1.30/unit) is not netted.</t>
+          <t>Prices here are from the audit read (24 Sep). The engine moved 15 bids and modifiers on 24 Sep after the audit, so where the live price differs, apply the step % to the live price and cap at the stop.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Top-of-search conversion follows the framework: under 15 TOS clicks in 90 days the group rate (or the product rate where the group has under 50 clicks); 15–49 with an order a click-weighted blend; 50+ the campaign’s own.</t>
+          <t>Deal stop = 3 × deal contribution × the campaign’s top-of-search conversion rate (the corrections doc’s loss stop, recomputed at the deal price). Deal contribution = deal price − 15% referral − FBA fee − landed cost (Command Center economics); Amazon’s deal fee (~$1.30/unit) is not netted.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Step = the corrections doc’s delivery gap on the last 14 days: under 30% of required TOS clicks +30%, 30–70% +20%, over 70% +10%, at requirement none; no requirement on file +20%. Impression share is not in this data: where share did not rise after the last step, HALVE the step.</t>
+          <t>Top-of-search conversion follows the framework: under 15 TOS clicks in 90 days the group rate (or the product rate where the group has under 50 clicks); 15–49 with an order a click-weighted blend; 50+ the campaign’s own.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Children follow Joseph’s ruling: push only “IN — push” children; hold flat on “hold bids”, “rides”, “OUT”. Budget: Joseph’s size envelopes (King ~$350/day, Queen ~$160, Full ~$60, Twin ~$10, Cal King unchanged).</t>
+          <t>Step = the corrections doc’s delivery gap on the last 14 days: under 30% of required TOS clicks +30%, 30–70% +20%, over 70% +10%, at requirement none; no requirement on file +20%. Impression share is not in this data: where share did not rise after the last step, HALVE the step.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Modifiers over 500% need human sign-off under the operator ruling of 9 Sep (900% is the hard cap); they are marked in Notes.</t>
+          <t>Children follow Joseph’s ruling: push only “IN — push” children; hold flat on “hold bids”, “rides”, “OUT”. Budget: Joseph’s size envelopes (King ~$350/day, Queen ~$160, Full ~$60, Twin ~$10, Cal King unchanged).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Budget rule during the deal: read budget use every morning and around midday; +30% the same day on any pushed campaign at 80%+ used. No other budget raises.</t>
+          <t>Modifiers over 500% need human sign-off under the operator ruling of 9 Sep (900% is the hard cap); they are marked in Notes.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Budget rule during the deal: read budget use every morning and around midday; +30% the same day on any pushed campaign at 80%+ used. No other budget raises.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Daily read to 30 Sep: TOS clicks, impression share, placement mix, budget use/hours out, Queen White stock, Bamboo|Queen and Bamboo|King median rank. Share rose → step again; flat → halve; at the stop → hold. Step-down review on 1–2 Oct, not 30 Sep.</t>
         </is>
@@ -965,7 +980,7 @@
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09); This campaign has engine rows on the pull list; this row replaces them</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep); This campaign has engine rows on the pull list; this row replaces them</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1098,7 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09)</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep)</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1205,7 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09)</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep)</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1312,7 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09)</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep)</t>
         </is>
       </c>
     </row>
@@ -1413,7 +1428,6 @@
       <c r="AC7" t="n">
         <v>4</v>
       </c>
-      <c r="AD7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1516,7 +1530,6 @@
       <c r="AC8" t="n">
         <v>8</v>
       </c>
-      <c r="AD8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1866,7 +1879,6 @@
       <c r="AC11" t="n">
         <v>0</v>
       </c>
-      <c r="AD11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2098,7 +2110,6 @@
       <c r="AC13" t="n">
         <v>0</v>
       </c>
-      <c r="AD13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2316,7 +2327,6 @@
       <c r="AC15" t="n">
         <v>10</v>
       </c>
-      <c r="AD15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2432,7 +2442,7 @@
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09)</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep)</t>
         </is>
       </c>
     </row>
@@ -2550,7 +2560,7 @@
       </c>
       <c r="AD17" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09); This campaign has engine rows on the pull list; this row replaces them</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep); This campaign has engine rows on the pull list; this row replaces them</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2667,7 @@
       </c>
       <c r="AD18" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09)</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep)</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2785,7 @@
       </c>
       <c r="AD19" t="inlineStr">
         <is>
-          <t>Past the 900% wall: base carries the rest (base = price ÷ 10); Modifier over the 500% working cap: human sign-off (operator 2026-09-09)</t>
+          <t>Past the 900% wall: base carries the rest (base = price ÷ 10); Modifier over 500%: APPROVED (operator sign-off 26 Sep)</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3021,7 @@
       </c>
       <c r="AD21" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09)</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep)</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3246,7 @@
       </c>
       <c r="AD23" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09)</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep)</t>
         </is>
       </c>
     </row>
@@ -3341,7 +3351,6 @@
       <c r="AC24" t="n">
         <v>1</v>
       </c>
-      <c r="AD24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3455,7 +3464,6 @@
       <c r="AC25" t="n">
         <v>2</v>
       </c>
-      <c r="AD25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3569,7 +3577,6 @@
       <c r="AC26" t="n">
         <v>1</v>
       </c>
-      <c r="AD26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3672,7 +3679,6 @@
       <c r="AC27" t="n">
         <v>1</v>
       </c>
-      <c r="AD27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3904,7 +3910,6 @@
       <c r="AC29" t="n">
         <v>0</v>
       </c>
-      <c r="AD29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4125,7 +4130,6 @@
       <c r="AC31" t="n">
         <v>0</v>
       </c>
-      <c r="AD31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4228,7 +4232,6 @@
       <c r="AC32" t="n">
         <v>0</v>
       </c>
-      <c r="AD32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4342,7 +4345,6 @@
       <c r="AC33" t="n">
         <v>0</v>
       </c>
-      <c r="AD33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4675,7 +4677,6 @@
       <c r="AC36" t="n">
         <v>0</v>
       </c>
-      <c r="AD36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4791,7 +4792,7 @@
       </c>
       <c r="AD37" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09); Queen White: check stock every morning (Sellerboard 6.88/day vs 4.3 in the plan)</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep); Queen White: check stock every morning (Sellerboard 6.88/day vs 4.3 in the plan)</t>
         </is>
       </c>
     </row>
@@ -4909,7 +4910,7 @@
       </c>
       <c r="AD38" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09); Product pages 80% of 14-day clicks: base −25% in the same write; Queen White: check stock every morning (Sellerboard 6.88/day vs 4.3 in the plan)</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep); Product pages 80% of 14-day clicks: base −25% in the same write; Queen White: check stock every morning (Sellerboard 6.88/day vs 4.3 in the plan)</t>
         </is>
       </c>
     </row>
@@ -5132,7 +5133,6 @@
       <c r="AC40" t="n">
         <v>11</v>
       </c>
-      <c r="AD40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5471,7 +5471,6 @@
       <c r="AC43" t="n">
         <v>10</v>
       </c>
-      <c r="AD43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5705,7 +5704,7 @@
       </c>
       <c r="AD45" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09); Queen White: check stock every morning (Sellerboard 6.88/day vs 4.3 in the plan)</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep); Queen White: check stock every morning (Sellerboard 6.88/day vs 4.3 in the plan)</t>
         </is>
       </c>
     </row>
@@ -5941,7 +5940,7 @@
       </c>
       <c r="AD47" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09); Queen White: check stock every morning (Sellerboard 6.88/day vs 4.3 in the plan)</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep); Queen White: check stock every morning (Sellerboard 6.88/day vs 4.3 in the plan)</t>
         </is>
       </c>
     </row>
@@ -6402,7 +6401,7 @@
       </c>
       <c r="AD51" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09); Queen White: check stock every morning (Sellerboard 6.88/day vs 4.3 in the plan)</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep); Queen White: check stock every morning (Sellerboard 6.88/day vs 4.3 in the plan)</t>
         </is>
       </c>
     </row>
@@ -6638,7 +6637,7 @@
       </c>
       <c r="AD53" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09); Queen White: check stock every morning (Sellerboard 6.88/day vs 4.3 in the plan)</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep); Queen White: check stock every morning (Sellerboard 6.88/day vs 4.3 in the plan)</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6980,7 @@
       </c>
       <c r="AD56" t="inlineStr">
         <is>
-          <t>Modifier over the 500% working cap: human sign-off (operator 2026-09-09); Queen White: check stock every morning (Sellerboard 6.88/day vs 4.3 in the plan)</t>
+          <t>Modifier over 500%: APPROVED (operator sign-off 26 Sep); Queen White: check stock every morning (Sellerboard 6.88/day vs 4.3 in the plan)</t>
         </is>
       </c>
     </row>
@@ -7908,7 +7907,7 @@
       </c>
       <c r="AD64" t="inlineStr">
         <is>
-          <t>Confirm enrolment first (Umair: could not enroll (zero safe allocation)); if not in the deal, hold flat; Modifier over the 500% working cap: human sign-off (operator 2026-09-09)</t>
+          <t>Confirm enrolment first (Umair: could not enroll (zero safe allocation)); if not in the deal, hold flat; Modifier over 500%: APPROVED (operator sign-off 26 Sep)</t>
         </is>
       </c>
     </row>
@@ -8144,7 +8143,7 @@
       </c>
       <c r="AD66" t="inlineStr">
         <is>
-          <t>Confirm enrolment first (Umair: could not enroll (zero safe allocation)); if not in the deal, hold flat; Modifier over the 500% working cap: human sign-off (operator 2026-09-09)</t>
+          <t>Confirm enrolment first (Umair: could not enroll (zero safe allocation)); if not in the deal, hold flat; Modifier over 500%: APPROVED (operator sign-off 26 Sep)</t>
         </is>
       </c>
     </row>
@@ -8478,7 +8477,6 @@
       <c r="AC69" t="n">
         <v>0</v>
       </c>
-      <c r="AD69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -8577,7 +8575,6 @@
       <c r="AC70" t="n">
         <v>0</v>
       </c>
-      <c r="AD70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8665,7 +8662,6 @@
       <c r="AC71" t="n">
         <v>0</v>
       </c>
-      <c r="AD71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -8781,7 +8777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -8802,148 +8798,100 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>CHOSEN 26 Sep: OPTION A. Option B is kept only as a fallback if the first deal days read weak, and only with Erik’s approval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Campaign</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Flagship</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Advertised child</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Deal ruling</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>TOS clicks 90d</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>TOS CVR 90d %</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Bar (3× market) %</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>TOS price now</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Deal stop</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>Option A — as the doc says (+10% test; flagship flat)</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Option B — deal push (delivery-gap step, capped)</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>Step B</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>Spend/day 14d</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>DBS6-SP-Bamboo Sheet-(VHSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Bamboo</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>BAMBOO-KING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>IN — push</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1444</v>
-      </c>
-      <c r="G2" t="n">
-        <v>19.2</v>
-      </c>
-      <c r="H2" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="I2" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="J2" t="n">
-        <v>12.98</v>
-      </c>
-      <c r="K2" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="L2" t="n">
-        <v>7.93</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>+30%</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
-        <v>250</v>
-      </c>
-      <c r="O2" t="n">
-        <v>43.31</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DBS6-SP-Viscose Bamboo Sheets-[Bamboo]-(LSV)-Exact-(Ranking)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
+          <t>DBS6-SP-Bamboo Sheet-(VHSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>Bamboo</t>
@@ -8960,25 +8908,25 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>106</v>
+        <v>1444</v>
       </c>
       <c r="G3" t="n">
-        <v>17.9</v>
+        <v>19.2</v>
       </c>
       <c r="H3" t="n">
         <v>8.300000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>5.95</v>
+        <v>6.1</v>
       </c>
       <c r="J3" t="n">
-        <v>12.03</v>
+        <v>12.98</v>
       </c>
       <c r="K3" t="n">
-        <v>6.55</v>
+        <v>6.1</v>
       </c>
       <c r="L3" t="n">
-        <v>7.74</v>
+        <v>7.93</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -8986,19 +8934,18 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="O3" t="n">
-        <v>13.04</v>
+        <v>43.31</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DBS6-SP-Bamboo Sheets With Corner Straps-(VLSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
+          <t>DBS6-SP-Viscose Bamboo Sheets-[Bamboo]-(LSV)-Exact-(Ranking)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>Bamboo</t>
@@ -9015,25 +8962,25 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="G4" t="n">
-        <v>16.8</v>
+        <v>17.9</v>
       </c>
       <c r="H4" t="n">
         <v>8.300000000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>5.62</v>
+        <v>5.95</v>
       </c>
       <c r="J4" t="n">
-        <v>11.49</v>
+        <v>12.03</v>
       </c>
       <c r="K4" t="n">
-        <v>6.18</v>
+        <v>6.55</v>
       </c>
       <c r="L4" t="n">
-        <v>7.31</v>
+        <v>7.74</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -9041,19 +8988,18 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="O4" t="n">
-        <v>5.36</v>
+        <v>13.04</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DBS6-SP-Bamboo Bed Sheet-(VLSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>DBS6-SP-Bamboo Sheets With Corner Straps-(VLSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>Bamboo</t>
@@ -9070,45 +9016,44 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G5" t="n">
-        <v>8.9</v>
+        <v>16.8</v>
       </c>
       <c r="H5" t="n">
         <v>8.300000000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>6.58</v>
+        <v>5.62</v>
       </c>
       <c r="J5" t="n">
-        <v>6.1</v>
+        <v>11.49</v>
       </c>
       <c r="K5" t="n">
-        <v>6.1</v>
+        <v>6.18</v>
       </c>
       <c r="L5" t="n">
-        <v>6.1</v>
+        <v>7.31</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>+20%</t>
+          <t>+30%</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="O5" t="n">
-        <v>3.84</v>
+        <v>5.36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DBS6-SP-Black Bamboo Sheets-(LSV)-Exact-(Ranking)-DO-BAMBOO-KING-BLACK-6PCS</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
+          <t>DBS6-SP-Bamboo Bed Sheet-(VLSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>Bamboo</t>
@@ -9116,117 +9061,115 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>BAMBOO-KING-BLACK-6PCS</t>
+          <t>BAMBOO-KING-WHITE-6PCS</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>OUT — stock</t>
+          <t>IN — push</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>159</v>
+        <v>112</v>
       </c>
       <c r="G6" t="n">
-        <v>9.4</v>
+        <v>8.9</v>
       </c>
       <c r="H6" t="n">
         <v>8.300000000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>4.82</v>
+        <v>6.58</v>
       </c>
       <c r="J6" t="n">
-        <v>6.45</v>
+        <v>6.1</v>
       </c>
       <c r="K6" t="n">
-        <v>4.82</v>
+        <v>6.1</v>
       </c>
       <c r="L6" t="n">
-        <v>4.82</v>
+        <v>6.1</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>0 (hold)</t>
+          <t>+20%</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="O6" t="n">
-        <v>2.41</v>
+        <v>3.84</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DBS6-SP-Cooling Bed Sheets King-[Cooling|King]-(LSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>DBS6-SP-Black Bamboo Sheets-(LSV)-Exact-(Ranking)-DO-BAMBOO-KING-BLACK-6PCS</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Cooling|King</t>
+          <t>Bamboo</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BAMBOO-KING-WHITE-6PCS</t>
+          <t>BAMBOO-KING-BLACK-6PCS</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>IN — push</t>
+          <t>OUT — stock</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>28</v>
+        <v>159</v>
       </c>
       <c r="G7" t="n">
-        <v>10.7</v>
+        <v>9.4</v>
       </c>
       <c r="H7" t="n">
-        <v>10.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I7" t="n">
-        <v>5.72</v>
+        <v>4.82</v>
       </c>
       <c r="J7" t="n">
-        <v>11.18</v>
+        <v>6.45</v>
       </c>
       <c r="K7" t="n">
-        <v>6.29</v>
+        <v>4.82</v>
       </c>
       <c r="L7" t="n">
-        <v>6.29</v>
+        <v>4.82</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>as option A (Cooling / Cal King: no deal money)</t>
+          <t>0 (hold)</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="O7" t="n">
-        <v>1.52</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DBS6-SP-Cooling Bedsheets-(VLSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
+          <t>DBS6-SP-Cooling Bed Sheets King-[Cooling|King]-(LSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cooling</t>
+          <t>Cooling|King</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>BAMBOO-QUEEN-WHITE-6PCS</t>
+          <t>BAMBOO-KING-WHITE-6PCS</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -9235,25 +9178,25 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="G8" t="n">
-        <v>15.2</v>
+        <v>10.7</v>
       </c>
       <c r="H8" t="n">
-        <v>8.4</v>
+        <v>10.5</v>
       </c>
       <c r="I8" t="n">
-        <v>5.43</v>
+        <v>5.72</v>
       </c>
       <c r="J8" t="n">
-        <v>11.02</v>
+        <v>11.18</v>
       </c>
       <c r="K8" t="n">
-        <v>5.97</v>
+        <v>6.29</v>
       </c>
       <c r="L8" t="n">
-        <v>5.97</v>
+        <v>6.29</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -9261,27 +9204,26 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>8.449999999999999</v>
+        <v>10</v>
       </c>
       <c r="O8" t="n">
-        <v>1.48</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DBS6-SP-Bamboo Cooling Sheets Full Size-[Cooling|Full]-(LSV)-Exact-(Ranking)-DO-BAMBOO-FULL-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
+          <t>DBS6-SP-Cooling Bedsheets-(VLSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cooling|Full</t>
+          <t>Cooling</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>BAMBOO-FULL-WHITE-6PCS</t>
+          <t>BAMBOO-QUEEN-WHITE-6PCS</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -9290,25 +9232,25 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="G9" t="n">
-        <v>15</v>
+        <v>15.2</v>
       </c>
       <c r="H9" t="n">
-        <v>12.4</v>
+        <v>8.4</v>
       </c>
       <c r="I9" t="n">
-        <v>8.619999999999999</v>
+        <v>5.43</v>
       </c>
       <c r="J9" t="n">
-        <v>10.18</v>
+        <v>11.02</v>
       </c>
       <c r="K9" t="n">
-        <v>9.48</v>
+        <v>5.97</v>
       </c>
       <c r="L9" t="n">
-        <v>9.48</v>
+        <v>5.97</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -9316,19 +9258,18 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>10</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="O9" t="n">
-        <v>1.46</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DBS6-SP-Cooling Bed Sheets Full Size-[Cooling|Full]-(LSV)-Exact-(Ranking)-DO-BAMBOO-FULL-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
+          <t>DBS6-SP-Bamboo Cooling Sheets Full Size-[Cooling|Full]-(LSV)-Exact-(Ranking)-DO-BAMBOO-FULL-WHITE-6PCS</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>Cooling|Full</t>
@@ -9345,25 +9286,25 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G10" t="n">
-        <v>18.8</v>
+        <v>15</v>
       </c>
       <c r="H10" t="n">
         <v>12.4</v>
       </c>
       <c r="I10" t="n">
-        <v>4.81</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>10.51</v>
+        <v>10.18</v>
       </c>
       <c r="K10" t="n">
-        <v>5.29</v>
+        <v>9.48</v>
       </c>
       <c r="L10" t="n">
-        <v>5.29</v>
+        <v>9.48</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -9374,24 +9315,23 @@
         <v>10</v>
       </c>
       <c r="O10" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DBS6-SP-Twin Sheets Bamboo-(VLSV)-Exact-(Ranking)-DO-BAMBOO-TWIN-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
+          <t>DBS6-SP-Cooling Bed Sheets Full Size-[Cooling|Full]-(LSV)-Exact-(Ranking)-DO-BAMBOO-FULL-WHITE-6PCS</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Bamboo|Twin</t>
+          <t>Cooling|Full</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-SAGE GREEN-6PCS</t>
+          <t>BAMBOO-FULL-WHITE-6PCS</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -9400,53 +9340,52 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G11" t="n">
-        <v>30.4</v>
+        <v>18.8</v>
       </c>
       <c r="H11" t="n">
-        <v>10.9</v>
+        <v>12.4</v>
       </c>
       <c r="I11" t="n">
-        <v>5.04</v>
+        <v>4.81</v>
       </c>
       <c r="J11" t="n">
-        <v>8.93</v>
+        <v>10.51</v>
       </c>
       <c r="K11" t="n">
-        <v>5.54</v>
+        <v>5.29</v>
       </c>
       <c r="L11" t="n">
-        <v>6.55</v>
+        <v>5.29</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>+30%</t>
+          <t>as option A (Cooling / Cal King: no deal money)</t>
         </is>
       </c>
       <c r="N11" t="n">
         <v>10</v>
       </c>
       <c r="O11" t="n">
-        <v>0.35</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DBS6-SP-Bamboo Sheets California King-(LSV)-Exact-(Ranking)-DO-BAMBOO-CALIFKING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
+          <t>DBS6-SP-Twin Sheets Bamboo-(VLSV)-Exact-(Ranking)-DO-BAMBOO-TWIN-WHITE-6PCS</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Bamboo|California King</t>
+          <t>Bamboo|Twin</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>BAMBOO-CALIFKING-WHITE-6PCS</t>
+          <t>BAMBOO-TWIN-SAGE GREEN-6PCS</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -9455,53 +9394,52 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>98</v>
+        <v>23</v>
       </c>
       <c r="G12" t="n">
-        <v>18.4</v>
+        <v>30.4</v>
       </c>
       <c r="H12" t="n">
-        <v>8.9</v>
+        <v>10.9</v>
       </c>
       <c r="I12" t="n">
-        <v>2.84</v>
+        <v>5.04</v>
       </c>
       <c r="J12" t="n">
-        <v>12.24</v>
+        <v>8.93</v>
       </c>
       <c r="K12" t="n">
-        <v>3.12</v>
+        <v>5.54</v>
       </c>
       <c r="L12" t="n">
-        <v>3.12</v>
+        <v>6.55</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>as option A (Cooling / Cal King: no deal money)</t>
+          <t>+30%</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="O12" t="n">
-        <v>0</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DBS6-SP-Bamboo Sheets Twin Size-[Bamboo|Twin]-(LSV)-Exact-(Ranking)-DO-BAMBOO-TWIN-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
+          <t>DBS6-SP-Bamboo Sheets California King-(LSV)-Exact-(Ranking)-DO-BAMBOO-CALIFKING-WHITE-6PCS</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Bamboo|Twin</t>
+          <t>Bamboo|California King</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>BAMBOO-TWIN-SAGE GREEN-6PCS</t>
+          <t>BAMBOO-CALIFKING-WHITE-6PCS</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -9510,33 +9448,33 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>27</v>
+        <v>98</v>
       </c>
       <c r="G13" t="n">
-        <v>11.1</v>
+        <v>18.4</v>
       </c>
       <c r="H13" t="n">
-        <v>10.9</v>
+        <v>8.9</v>
       </c>
       <c r="I13" t="n">
-        <v>1.35</v>
+        <v>2.84</v>
       </c>
       <c r="J13" t="n">
-        <v>6.57</v>
+        <v>12.24</v>
       </c>
       <c r="K13" t="n">
-        <v>1.49</v>
+        <v>3.12</v>
       </c>
       <c r="L13" t="n">
-        <v>1.62</v>
+        <v>3.12</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>+20%</t>
+          <t>as option A (Cooling / Cal King: no deal money)</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
@@ -9545,18 +9483,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DBS6-SP-Cooling Sheets Queen Deep Pockets-(VLSV)-Exact-(Ranking)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
+          <t>DBS6-SP-Bamboo Sheets Twin Size-[Bamboo|Twin]-(LSV)-Exact-(Ranking)-DO-BAMBOO-TWIN-WHITE-6PCS</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cooling|Queen</t>
+          <t>Bamboo|Twin</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>BAMBOO-QUEEN-WHITE-6PCS</t>
+          <t>BAMBOO-TWIN-SAGE GREEN-6PCS</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -9565,29 +9502,29 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G14" t="n">
-        <v>22.7</v>
+        <v>11.1</v>
       </c>
       <c r="H14" t="n">
-        <v>12.3</v>
+        <v>10.9</v>
       </c>
       <c r="I14" t="n">
-        <v>3.84</v>
+        <v>1.35</v>
       </c>
       <c r="J14" t="n">
-        <v>8.880000000000001</v>
+        <v>6.57</v>
       </c>
       <c r="K14" t="n">
-        <v>4.22</v>
+        <v>1.49</v>
       </c>
       <c r="L14" t="n">
-        <v>4.22</v>
+        <v>1.62</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>as option A (Cooling / Cal King: no deal money)</t>
+          <t>+20%</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -9600,18 +9537,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DBS6-SP-Cooling Sheets King Size Deep Pocket-[Cooling|King]-(LSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
+          <t>DBS6-SP-Cooling Sheets Queen Deep Pockets-(VLSV)-Exact-(Ranking)-DO-BAMBOO-QUEEN-WHITE-6PCS</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Cooling|King</t>
+          <t>Cooling|Queen</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>BAMBOO-KING-WHITE-6PCS</t>
+          <t>BAMBOO-QUEEN-WHITE-6PCS</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -9620,25 +9556,25 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G15" t="n">
-        <v>18.5</v>
+        <v>22.7</v>
       </c>
       <c r="H15" t="n">
-        <v>10.5</v>
+        <v>12.3</v>
       </c>
       <c r="I15" t="n">
-        <v>3.34</v>
+        <v>3.84</v>
       </c>
       <c r="J15" t="n">
-        <v>13.18</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>3.67</v>
+        <v>4.22</v>
       </c>
       <c r="L15" t="n">
-        <v>3.67</v>
+        <v>4.22</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -9646,7 +9582,7 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
@@ -9655,10 +9591,9 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DBS6-SP- cooling king size sheets-(VLSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
+          <t>DBS6-SP-Cooling Sheets King Size Deep Pocket-[Cooling|King]-(LSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>Cooling|King</t>
@@ -9675,25 +9610,25 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="G16" t="n">
-        <v>23.1</v>
+        <v>18.5</v>
       </c>
       <c r="H16" t="n">
         <v>10.5</v>
       </c>
       <c r="I16" t="n">
-        <v>5.19</v>
+        <v>3.34</v>
       </c>
       <c r="J16" t="n">
-        <v>15.77</v>
+        <v>13.18</v>
       </c>
       <c r="K16" t="n">
-        <v>5.71</v>
+        <v>3.67</v>
       </c>
       <c r="L16" t="n">
-        <v>5.71</v>
+        <v>3.67</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -9701,7 +9636,7 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>8.449999999999999</v>
+        <v>5</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
@@ -9710,18 +9645,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DBS6-SP-California King Sheets Bamboo-(VLSV)-Exact-(Ranking)-DO-BAMBOO-CALIFKING-WHITE-6PCS</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
+          <t>DBS6-SP- cooling king size sheets-(VLSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Bamboo|California King</t>
+          <t>Cooling|King</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>BAMBOO-CALIFKING-WHITE-6PCS</t>
+          <t>BAMBOO-KING-WHITE-6PCS</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -9730,25 +9664,25 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="G17" t="n">
-        <v>18.8</v>
+        <v>23.1</v>
       </c>
       <c r="H17" t="n">
-        <v>8.9</v>
+        <v>10.5</v>
       </c>
       <c r="I17" t="n">
-        <v>4.96</v>
+        <v>5.19</v>
       </c>
       <c r="J17" t="n">
-        <v>11</v>
+        <v>15.77</v>
       </c>
       <c r="K17" t="n">
-        <v>5.46</v>
+        <v>5.71</v>
       </c>
       <c r="L17" t="n">
-        <v>5.46</v>
+        <v>5.71</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -9756,7 +9690,7 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>90</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
@@ -9765,60 +9699,114 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>DBS6-SP-California King Sheets Bamboo-(VLSV)-Exact-(Ranking)-DO-BAMBOO-CALIFKING-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Bamboo|California King</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>BAMBOO-CALIFKING-WHITE-6PCS</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>IN — push</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>16</v>
+      </c>
+      <c r="G18" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="H18" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="I18" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="J18" t="n">
+        <v>11</v>
+      </c>
+      <c r="K18" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="L18" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>as option A (Cooling / Cal King: no deal money)</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>90</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>DBS6-SP-Cooling Sheets For Hot Sleepers-(VLSV)-Exact-(Ranking)-DO-BAMBOO-KING-WHITE-6PCS</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Cooling</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>BAMBOO-KING-WHITE-6PCS</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>IN — push</t>
         </is>
       </c>
-      <c r="F18" t="n">
+      <c r="F19" t="n">
         <v>49</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G19" t="n">
         <v>22.4</v>
       </c>
-      <c r="H18" t="n">
+      <c r="H19" t="n">
         <v>8.4</v>
       </c>
-      <c r="I18" t="n">
+      <c r="I19" t="n">
         <v>4.29</v>
       </c>
-      <c r="J18" t="n">
+      <c r="J19" t="n">
         <v>15.22</v>
       </c>
-      <c r="K18" t="n">
+      <c r="K19" t="n">
         <v>4.72</v>
       </c>
-      <c r="L18" t="n">
+      <c r="L19" t="n">
         <v>4.72</v>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>as option A (Cooling / Cal King: no deal money)</t>
         </is>
       </c>
-      <c r="N18" t="n">
+      <c r="N19" t="n">
         <v>20</v>
       </c>
-      <c r="O18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Decision needed from Erik/Joseph: Option A keeps the operator rulings (flagship flat, out-of-focus +10% test for two weeks). Option B pushes King and Queen converters for the 5 deal days, capped at the deal stop, then returns to Option A on 1 Oct. Children not “IN — push” stay flat under either option.</t>
         </is>
@@ -11766,7 +11754,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -11799,7 +11786,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
         <v>84.98999999999999</v>
       </c>
@@ -11832,7 +11818,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -11871,7 +11856,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>80.73999999999999</v>
       </c>
@@ -11910,7 +11894,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -11943,7 +11926,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -11982,7 +11964,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
         <v>80.98999999999999</v>
       </c>
@@ -12021,7 +12002,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -12060,7 +12040,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -12099,7 +12078,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -12138,7 +12116,6 @@
           <t>OUT — stock</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -12177,7 +12154,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -12216,7 +12192,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -12255,7 +12230,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -12288,7 +12262,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -12327,7 +12300,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -12409,7 +12381,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
         <v>62.99</v>
       </c>
@@ -12442,7 +12413,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
         <v>62.99</v>
       </c>
@@ -12475,7 +12445,6 @@
           <t>IN — rides (don’t advertise)</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
         <v>67.48999999999999</v>
       </c>
@@ -12514,7 +12483,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
         <v>57.36</v>
       </c>
@@ -12553,7 +12521,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
         <v>62.99</v>
       </c>
@@ -12592,7 +12559,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
         <v>62.99</v>
       </c>
@@ -12631,7 +12597,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
         <v>62.99</v>
       </c>
@@ -12670,7 +12635,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
         <v>62.99</v>
       </c>
@@ -12709,7 +12673,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
         <v>62.99</v>
       </c>
@@ -12742,7 +12705,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
         <v>62.99</v>
       </c>
@@ -12781,7 +12743,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
         <v>62.99</v>
       </c>
@@ -12814,7 +12775,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
         <v>62.99</v>
       </c>
@@ -12853,7 +12813,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="n">
         <v>69.98999999999999</v>
       </c>
@@ -12892,7 +12851,6 @@
           <t>OUT — stock</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
         <v>62.99</v>
       </c>
@@ -12931,7 +12889,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
         <v>62.99</v>
       </c>
@@ -12970,7 +12927,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
         <v>62.99</v>
       </c>
@@ -13009,7 +12965,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="n">
         <v>62.99</v>
       </c>
@@ -13048,7 +13003,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="n">
         <v>62.99</v>
       </c>
@@ -13081,7 +13035,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
         <v>62.99</v>
       </c>
@@ -13120,7 +13073,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
         <v>62.99</v>
       </c>
@@ -13159,7 +13111,6 @@
           <t>OUT — stock</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -13198,7 +13149,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
         <v>84.98999999999999</v>
       </c>
@@ -13231,7 +13181,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -13270,7 +13219,6 @@
           <t>IN — rides (don’t advertise)</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
         <v>80.73999999999999</v>
       </c>
@@ -13309,7 +13257,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -13348,7 +13295,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="n">
         <v>75.98999999999999</v>
       </c>
@@ -13387,7 +13333,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -13426,7 +13371,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="n">
         <v>75.98999999999999</v>
       </c>
@@ -13465,7 +13409,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -13504,7 +13447,6 @@
           <t>IN — hold bids</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -13543,7 +13485,6 @@
           <t>IN — hold bids</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -13582,7 +13523,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -13621,7 +13561,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
         <v>68.39</v>
       </c>
@@ -13660,7 +13599,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
         <v>80.73999999999999</v>
       </c>
@@ -13742,7 +13680,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="n">
         <v>76.48999999999999</v>
       </c>
@@ -13781,7 +13718,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" t="n">
         <v>71.98999999999999</v>
       </c>
@@ -13820,7 +13756,6 @@
           <t>OUT — stock</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="n">
         <v>71.98999999999999</v>
       </c>
@@ -13859,7 +13794,6 @@
           <t>IN — hold bids</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
       <c r="E57" t="n">
         <v>72.23999999999999</v>
       </c>
@@ -13941,7 +13875,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="n">
         <v>72.23999999999999</v>
       </c>
@@ -13980,7 +13913,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="n">
         <v>71.98999999999999</v>
       </c>
@@ -14019,7 +13951,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="n">
         <v>71.98999999999999</v>
       </c>
@@ -14058,7 +13989,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="n">
         <v>71.23999999999999</v>
       </c>
@@ -14097,7 +14027,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="n">
         <v>71.23999999999999</v>
       </c>
@@ -14136,7 +14065,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
       <c r="E64" t="n">
         <v>71.23999999999999</v>
       </c>
@@ -14175,7 +14103,6 @@
           <t>IN — rides (don’t advertise)</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="n">
         <v>72.23999999999999</v>
       </c>
@@ -14214,7 +14141,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
       <c r="E66" t="n">
         <v>71.98999999999999</v>
       </c>
@@ -14253,7 +14179,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
       <c r="E67" t="n">
         <v>71.98999999999999</v>
       </c>
@@ -14286,7 +14211,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
       <c r="E68" t="n">
         <v>71.98999999999999</v>
       </c>
@@ -14319,7 +14243,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
       <c r="E69" t="n">
         <v>71.23999999999999</v>
       </c>
@@ -14358,7 +14281,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr"/>
       <c r="E70" t="n">
         <v>71.98999999999999</v>
       </c>
@@ -14397,7 +14319,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="n">
         <v>71.98999999999999</v>
       </c>
@@ -14436,7 +14357,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
       <c r="E72" t="n">
         <v>53.99</v>
       </c>
@@ -14469,7 +14389,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr"/>
       <c r="E73" t="n">
         <v>53.99</v>
       </c>
@@ -14508,7 +14427,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
       <c r="E74" t="n">
         <v>53.99</v>
       </c>
@@ -14547,7 +14465,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
       <c r="E75" t="n">
         <v>53.99</v>
       </c>
@@ -14586,7 +14503,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
       <c r="E76" t="n">
         <v>53.99</v>
       </c>
@@ -14625,7 +14541,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" t="n">
         <v>53.99</v>
       </c>
@@ -14658,7 +14573,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr"/>
       <c r="E78" t="n">
         <v>53.99</v>
       </c>
@@ -14697,7 +14611,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
       <c r="E79" t="n">
         <v>53.99</v>
       </c>
@@ -14736,7 +14649,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
       <c r="E80" t="n">
         <v>53.99</v>
       </c>
@@ -14775,7 +14687,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr"/>
       <c r="E81" t="n">
         <v>52.64</v>
       </c>
@@ -14814,7 +14725,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr"/>
       <c r="E82" t="n">
         <v>53.99</v>
       </c>
@@ -14853,7 +14763,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr"/>
       <c r="E83" t="n">
         <v>59.99</v>
       </c>
@@ -14892,7 +14801,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
       <c r="E84" t="n">
         <v>58.49</v>
       </c>
@@ -14931,7 +14839,6 @@
           <t>IN — push</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr"/>
       <c r="E85" t="n">
         <v>53.99</v>
       </c>
@@ -15013,7 +14920,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
       <c r="E87" t="n">
         <v>53.99</v>
       </c>
@@ -15052,7 +14958,6 @@
           <t>OUT — no stock / not in deal</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
       <c r="E88" t="n">
         <v>53.99</v>
       </c>
@@ -15213,7 +15118,6 @@
           <t>unchanged</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>0</v>
       </c>

</xml_diff>